<commit_message>
fix: melhorias pylint — docstrings, trailing whitespace, f-strings
</commit_message>
<xml_diff>
--- a/data/resultados.xlsx
+++ b/data/resultados.xlsx
@@ -722,7 +722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -795,1505 +795,1247 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Distrito 10</t>
+          <t>Aveiro</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>85330</v>
+        <v>63271</v>
       </c>
       <c r="C2" t="n">
-        <v>81644</v>
+        <v>62427</v>
       </c>
       <c r="D2" t="n">
-        <v>274104</v>
+        <v>206065</v>
       </c>
       <c r="E2" t="n">
-        <v>246334</v>
+        <v>218648</v>
       </c>
       <c r="F2" t="n">
-        <v>276068</v>
+        <v>202071</v>
       </c>
       <c r="G2" t="n">
-        <v>256466</v>
+        <v>189070</v>
       </c>
       <c r="H2" t="n">
-        <v>276055</v>
+        <v>204174</v>
       </c>
       <c r="I2" t="n">
-        <v>292020</v>
+        <v>224217</v>
       </c>
       <c r="J2" t="n">
-        <v>255906</v>
+        <v>176196</v>
       </c>
       <c r="K2" t="n">
-        <v>271444</v>
+        <v>201517</v>
       </c>
       <c r="L2" t="n">
-        <v>302388</v>
+        <v>198162</v>
       </c>
       <c r="M2" t="n">
-        <v>267564</v>
+        <v>216752</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Distrito 11</t>
+          <t>Beja</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>84262</v>
+        <v>31454</v>
       </c>
       <c r="C3" t="n">
-        <v>83035</v>
+        <v>31860</v>
       </c>
       <c r="D3" t="n">
-        <v>267975</v>
+        <v>102525</v>
       </c>
       <c r="E3" t="n">
-        <v>288668</v>
+        <v>98210</v>
       </c>
       <c r="F3" t="n">
-        <v>240474</v>
+        <v>93466</v>
       </c>
       <c r="G3" t="n">
-        <v>282533</v>
+        <v>98732</v>
       </c>
       <c r="H3" t="n">
-        <v>262278</v>
+        <v>96169</v>
       </c>
       <c r="I3" t="n">
-        <v>270020</v>
+        <v>97064</v>
       </c>
       <c r="J3" t="n">
-        <v>242247</v>
+        <v>101825</v>
       </c>
       <c r="K3" t="n">
-        <v>244801</v>
+        <v>106494</v>
       </c>
       <c r="L3" t="n">
-        <v>238243</v>
+        <v>122182</v>
       </c>
       <c r="M3" t="n">
-        <v>294001</v>
+        <v>105548</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Distrito 20</t>
+          <t>Braga</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>21080</v>
+        <v>144891</v>
       </c>
       <c r="C4" t="n">
-        <v>19908</v>
+        <v>143103</v>
       </c>
       <c r="D4" t="n">
-        <v>65915</v>
+        <v>449773</v>
       </c>
       <c r="E4" t="n">
-        <v>61259</v>
+        <v>475718</v>
       </c>
       <c r="F4" t="n">
-        <v>67611</v>
+        <v>473398</v>
       </c>
       <c r="G4" t="n">
-        <v>64436</v>
+        <v>429806</v>
       </c>
       <c r="H4" t="n">
-        <v>60404</v>
+        <v>453932</v>
       </c>
       <c r="I4" t="n">
-        <v>62149</v>
+        <v>452757</v>
       </c>
       <c r="J4" t="n">
-        <v>55187</v>
+        <v>447666</v>
       </c>
       <c r="K4" t="n">
-        <v>60083</v>
+        <v>431216</v>
       </c>
       <c r="L4" t="n">
-        <v>74632</v>
+        <v>441505</v>
       </c>
       <c r="M4" t="n">
-        <v>76748</v>
+        <v>477845</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Distrito 21</t>
+          <t>Bragança</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>10374</v>
+        <v>101728</v>
       </c>
       <c r="C5" t="n">
-        <v>11952</v>
+        <v>103786</v>
       </c>
       <c r="D5" t="n">
-        <v>36610</v>
+        <v>336619</v>
       </c>
       <c r="E5" t="n">
-        <v>36951</v>
+        <v>314540</v>
       </c>
       <c r="F5" t="n">
-        <v>25855</v>
+        <v>327702</v>
       </c>
       <c r="G5" t="n">
-        <v>34296</v>
+        <v>322933</v>
       </c>
       <c r="H5" t="n">
-        <v>35765</v>
+        <v>323755</v>
       </c>
       <c r="I5" t="n">
-        <v>34915</v>
+        <v>336321</v>
       </c>
       <c r="J5" t="n">
-        <v>46638</v>
+        <v>346605</v>
       </c>
       <c r="K5" t="n">
-        <v>46411</v>
+        <v>334469</v>
       </c>
       <c r="L5" t="n">
-        <v>47550</v>
+        <v>345638</v>
       </c>
       <c r="M5" t="n">
-        <v>28800</v>
+        <v>360847</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Distrito 30</t>
+          <t>Castelo Branco</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>97983</v>
+        <v>51361</v>
       </c>
       <c r="C6" t="n">
-        <v>100631</v>
+        <v>53970</v>
       </c>
       <c r="D6" t="n">
-        <v>315619</v>
+        <v>167344</v>
       </c>
       <c r="E6" t="n">
-        <v>331759</v>
+        <v>166585</v>
       </c>
       <c r="F6" t="n">
-        <v>337048</v>
+        <v>186499</v>
       </c>
       <c r="G6" t="n">
-        <v>301684</v>
+        <v>171035</v>
       </c>
       <c r="H6" t="n">
-        <v>310879</v>
+        <v>182219</v>
       </c>
       <c r="I6" t="n">
-        <v>312941</v>
+        <v>159932</v>
       </c>
       <c r="J6" t="n">
-        <v>293848</v>
+        <v>169611</v>
       </c>
       <c r="K6" t="n">
-        <v>313490</v>
+        <v>164342</v>
       </c>
       <c r="L6" t="n">
-        <v>307413</v>
+        <v>168112</v>
       </c>
       <c r="M6" t="n">
-        <v>323935</v>
+        <v>169165</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Distrito 03</t>
+          <t>Coimbra</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2774</v>
+        <v>67813</v>
       </c>
       <c r="C7" t="n">
-        <v>2069</v>
+        <v>70516</v>
       </c>
       <c r="D7" t="n">
-        <v>7070</v>
+        <v>218154</v>
       </c>
       <c r="E7" t="n">
-        <v>6169</v>
+        <v>225717</v>
       </c>
       <c r="F7" t="n">
-        <v>7088</v>
+        <v>206571</v>
       </c>
       <c r="G7" t="n">
-        <v>4699</v>
+        <v>205048</v>
       </c>
       <c r="H7" t="n">
-        <v>7110</v>
+        <v>202081</v>
       </c>
       <c r="I7" t="n">
-        <v>5597</v>
+        <v>213519</v>
       </c>
       <c r="J7" t="n">
-        <v>6621</v>
+        <v>195606</v>
       </c>
       <c r="K7" t="n">
-        <v>7927</v>
+        <v>219772</v>
       </c>
       <c r="L7" t="n">
-        <v>10075</v>
+        <v>223659</v>
       </c>
       <c r="M7" t="n">
-        <v>11872</v>
+        <v>228015</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Distrito 31</t>
+          <t>Évora</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>69386</v>
+        <v>30961</v>
       </c>
       <c r="C8" t="n">
-        <v>64564</v>
+        <v>27522</v>
       </c>
       <c r="D8" t="n">
-        <v>210723</v>
+        <v>116762</v>
       </c>
       <c r="E8" t="n">
-        <v>208112</v>
+        <v>88493</v>
       </c>
       <c r="F8" t="n">
-        <v>201002</v>
+        <v>106294</v>
       </c>
       <c r="G8" t="n">
-        <v>200419</v>
+        <v>94024</v>
       </c>
       <c r="H8" t="n">
-        <v>222443</v>
+        <v>86171</v>
       </c>
       <c r="I8" t="n">
-        <v>208383</v>
+        <v>98443</v>
       </c>
       <c r="J8" t="n">
-        <v>224446</v>
+        <v>86106</v>
       </c>
       <c r="K8" t="n">
-        <v>183977</v>
+        <v>94345</v>
       </c>
       <c r="L8" t="n">
-        <v>200797</v>
+        <v>78678</v>
       </c>
       <c r="M8" t="n">
-        <v>228498</v>
+        <v>83136</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Distrito 40</t>
+          <t>Faro</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>83040</v>
+        <v>31656</v>
       </c>
       <c r="C9" t="n">
-        <v>81163</v>
+        <v>28731</v>
       </c>
       <c r="D9" t="n">
-        <v>265070</v>
+        <v>85980</v>
       </c>
       <c r="E9" t="n">
-        <v>244287</v>
+        <v>91369</v>
       </c>
       <c r="F9" t="n">
-        <v>268926</v>
+        <v>89556</v>
       </c>
       <c r="G9" t="n">
-        <v>259442</v>
+        <v>96904</v>
       </c>
       <c r="H9" t="n">
-        <v>261280</v>
+        <v>91444</v>
       </c>
       <c r="I9" t="n">
-        <v>259713</v>
+        <v>86203</v>
       </c>
       <c r="J9" t="n">
-        <v>273700</v>
+        <v>94405</v>
       </c>
       <c r="K9" t="n">
-        <v>269878</v>
+        <v>93269</v>
       </c>
       <c r="L9" t="n">
-        <v>275021</v>
+        <v>87241</v>
       </c>
       <c r="M9" t="n">
-        <v>286826</v>
+        <v>98257</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Distrito 41</t>
+          <t>Guarda</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>21962</v>
+        <v>107203</v>
       </c>
       <c r="C10" t="n">
-        <v>24479</v>
+        <v>108019</v>
       </c>
       <c r="D10" t="n">
-        <v>82119</v>
+        <v>342578</v>
       </c>
       <c r="E10" t="n">
-        <v>78735</v>
+        <v>332321</v>
       </c>
       <c r="F10" t="n">
-        <v>63085</v>
+        <v>307390</v>
       </c>
       <c r="G10" t="n">
-        <v>70800</v>
+        <v>346689</v>
       </c>
       <c r="H10" t="n">
-        <v>69122</v>
+        <v>322905</v>
       </c>
       <c r="I10" t="n">
-        <v>84184</v>
+        <v>357229</v>
       </c>
       <c r="J10" t="n">
-        <v>79030</v>
+        <v>347264</v>
       </c>
       <c r="K10" t="n">
-        <v>75294</v>
+        <v>345931</v>
       </c>
       <c r="L10" t="n">
-        <v>76907</v>
+        <v>349694</v>
       </c>
       <c r="M10" t="n">
-        <v>82417</v>
+        <v>338486</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Distrito 50</t>
+          <t>Leiria</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>47285</v>
+        <v>49264</v>
       </c>
       <c r="C11" t="n">
-        <v>48645</v>
+        <v>46769</v>
       </c>
       <c r="D11" t="n">
-        <v>154312</v>
+        <v>152258</v>
       </c>
       <c r="E11" t="n">
-        <v>148527</v>
+        <v>128431</v>
       </c>
       <c r="F11" t="n">
-        <v>175000</v>
+        <v>146919</v>
       </c>
       <c r="G11" t="n">
-        <v>153991</v>
+        <v>148401</v>
       </c>
       <c r="H11" t="n">
-        <v>169206</v>
+        <v>155502</v>
       </c>
       <c r="I11" t="n">
-        <v>149131</v>
+        <v>151609</v>
       </c>
       <c r="J11" t="n">
-        <v>157354</v>
+        <v>145036</v>
       </c>
       <c r="K11" t="n">
-        <v>149390</v>
+        <v>143831</v>
       </c>
       <c r="L11" t="n">
-        <v>153988</v>
+        <v>178553</v>
       </c>
       <c r="M11" t="n">
-        <v>157808</v>
+        <v>153573</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Distrito 51</t>
+          <t>Lisboa</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4076</v>
+        <v>57057</v>
       </c>
       <c r="C12" t="n">
-        <v>5325</v>
+        <v>55483</v>
       </c>
       <c r="D12" t="n">
-        <v>13032</v>
+        <v>183756</v>
       </c>
       <c r="E12" t="n">
-        <v>18058</v>
+        <v>187923</v>
       </c>
       <c r="F12" t="n">
-        <v>11499</v>
+        <v>167552</v>
       </c>
       <c r="G12" t="n">
-        <v>17044</v>
+        <v>201528</v>
       </c>
       <c r="H12" t="n">
-        <v>13013</v>
+        <v>178657</v>
       </c>
       <c r="I12" t="n">
-        <v>10801</v>
+        <v>186214</v>
       </c>
       <c r="J12" t="n">
-        <v>12257</v>
+        <v>176921</v>
       </c>
       <c r="K12" t="n">
-        <v>14952</v>
+        <v>170897</v>
       </c>
       <c r="L12" t="n">
-        <v>14124</v>
+        <v>163916</v>
       </c>
       <c r="M12" t="n">
-        <v>11357</v>
+        <v>191240</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Distrito 60</t>
+          <t>Portalegre</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>39136</v>
+        <v>28750</v>
       </c>
       <c r="C13" t="n">
-        <v>39115</v>
+        <v>31133</v>
       </c>
       <c r="D13" t="n">
-        <v>120467</v>
+        <v>96156</v>
       </c>
       <c r="E13" t="n">
-        <v>120782</v>
+        <v>93479</v>
       </c>
       <c r="F13" t="n">
-        <v>106788</v>
+        <v>82990</v>
       </c>
       <c r="G13" t="n">
-        <v>113618</v>
+        <v>80639</v>
       </c>
       <c r="H13" t="n">
-        <v>114346</v>
+        <v>89399</v>
       </c>
       <c r="I13" t="n">
-        <v>119083</v>
+        <v>95963</v>
       </c>
       <c r="J13" t="n">
-        <v>109440</v>
+        <v>90764</v>
       </c>
       <c r="K13" t="n">
-        <v>122352</v>
+        <v>91850</v>
       </c>
       <c r="L13" t="n">
-        <v>125769</v>
+        <v>103786</v>
       </c>
       <c r="M13" t="n">
-        <v>121833</v>
+        <v>95663</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Distrito 61</t>
+          <t>Porto</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>28677</v>
+        <v>107340</v>
       </c>
       <c r="C14" t="n">
-        <v>31401</v>
+        <v>113242</v>
       </c>
       <c r="D14" t="n">
-        <v>97687</v>
+        <v>330232</v>
       </c>
       <c r="E14" t="n">
-        <v>104935</v>
+        <v>338714</v>
       </c>
       <c r="F14" t="n">
-        <v>99783</v>
+        <v>360341</v>
       </c>
       <c r="G14" t="n">
-        <v>91430</v>
+        <v>346037</v>
       </c>
       <c r="H14" t="n">
-        <v>87735</v>
+        <v>340447</v>
       </c>
       <c r="I14" t="n">
-        <v>94436</v>
+        <v>331960</v>
       </c>
       <c r="J14" t="n">
-        <v>86166</v>
+        <v>333167</v>
       </c>
       <c r="K14" t="n">
-        <v>97420</v>
+        <v>347477</v>
       </c>
       <c r="L14" t="n">
-        <v>97890</v>
+        <v>329431</v>
       </c>
       <c r="M14" t="n">
-        <v>106182</v>
+        <v>348478</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Distrito 70</t>
+          <t>Santarém</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>23971</v>
+        <v>57277</v>
       </c>
       <c r="C15" t="n">
-        <v>21059</v>
+        <v>56747</v>
       </c>
       <c r="D15" t="n">
-        <v>90869</v>
+        <v>198538</v>
       </c>
       <c r="E15" t="n">
-        <v>68045</v>
+        <v>168775</v>
       </c>
       <c r="F15" t="n">
-        <v>83948</v>
+        <v>179813</v>
       </c>
       <c r="G15" t="n">
-        <v>75605</v>
+        <v>186307</v>
       </c>
       <c r="H15" t="n">
-        <v>67698</v>
+        <v>198269</v>
       </c>
       <c r="I15" t="n">
-        <v>79548</v>
+        <v>173266</v>
       </c>
       <c r="J15" t="n">
-        <v>63051</v>
+        <v>167270</v>
       </c>
       <c r="K15" t="n">
-        <v>75744</v>
+        <v>196003</v>
       </c>
       <c r="L15" t="n">
-        <v>62793</v>
+        <v>177598</v>
       </c>
       <c r="M15" t="n">
-        <v>64556</v>
+        <v>170772</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Distrito 71</t>
+          <t>Setúbal</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>6990</v>
+        <v>22646</v>
       </c>
       <c r="C16" t="n">
-        <v>6463</v>
+        <v>25203</v>
       </c>
       <c r="D16" t="n">
-        <v>25893</v>
+        <v>69689</v>
       </c>
       <c r="E16" t="n">
-        <v>20448</v>
+        <v>76771</v>
       </c>
       <c r="F16" t="n">
-        <v>22346</v>
+        <v>84251</v>
       </c>
       <c r="G16" t="n">
-        <v>18419</v>
+        <v>77634</v>
       </c>
       <c r="H16" t="n">
-        <v>18473</v>
+        <v>83946</v>
       </c>
       <c r="I16" t="n">
-        <v>18895</v>
+        <v>68435</v>
       </c>
       <c r="J16" t="n">
-        <v>23055</v>
+        <v>80472</v>
       </c>
       <c r="K16" t="n">
-        <v>18601</v>
+        <v>83897</v>
       </c>
       <c r="L16" t="n">
-        <v>15885</v>
+        <v>81842</v>
       </c>
       <c r="M16" t="n">
-        <v>18580</v>
+        <v>74533</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Distrito 80</t>
+          <t>Viana do Castelo</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>19021</v>
+        <v>86084</v>
       </c>
       <c r="C17" t="n">
-        <v>16570</v>
+        <v>85910</v>
       </c>
       <c r="D17" t="n">
-        <v>49181</v>
+        <v>325287</v>
       </c>
       <c r="E17" t="n">
-        <v>55760</v>
+        <v>265964</v>
       </c>
       <c r="F17" t="n">
-        <v>50522</v>
+        <v>263424</v>
       </c>
       <c r="G17" t="n">
-        <v>64495</v>
+        <v>288513</v>
       </c>
       <c r="H17" t="n">
-        <v>54027</v>
+        <v>293656</v>
       </c>
       <c r="I17" t="n">
-        <v>53751</v>
+        <v>276578</v>
       </c>
       <c r="J17" t="n">
-        <v>54813</v>
+        <v>288957</v>
       </c>
       <c r="K17" t="n">
-        <v>55318</v>
+        <v>295905</v>
       </c>
       <c r="L17" t="n">
-        <v>55038</v>
+        <v>276817</v>
       </c>
       <c r="M17" t="n">
-        <v>57583</v>
+        <v>303974</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Distrito 81</t>
+          <t>Vila Real</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>12635</v>
+        <v>82448</v>
       </c>
       <c r="C18" t="n">
-        <v>12161</v>
+        <v>86693</v>
       </c>
       <c r="D18" t="n">
-        <v>36799</v>
+        <v>246497</v>
       </c>
       <c r="E18" t="n">
-        <v>35609</v>
+        <v>245314</v>
       </c>
       <c r="F18" t="n">
-        <v>39034</v>
+        <v>260576</v>
       </c>
       <c r="G18" t="n">
-        <v>32409</v>
+        <v>261959</v>
       </c>
       <c r="H18" t="n">
-        <v>37417</v>
+        <v>235936</v>
       </c>
       <c r="I18" t="n">
-        <v>32452</v>
+        <v>258301</v>
       </c>
       <c r="J18" t="n">
-        <v>39592</v>
+        <v>267372</v>
       </c>
       <c r="K18" t="n">
-        <v>37951</v>
+        <v>267649</v>
       </c>
       <c r="L18" t="n">
-        <v>32203</v>
+        <v>269690</v>
       </c>
       <c r="M18" t="n">
-        <v>40674</v>
+        <v>295538</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Distrito 90</t>
+          <t>Viseu</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>59218</v>
+        <v>130124</v>
       </c>
       <c r="C19" t="n">
-        <v>60567</v>
+        <v>125511</v>
       </c>
       <c r="D19" t="n">
-        <v>192225</v>
+        <v>399668</v>
       </c>
       <c r="E19" t="n">
-        <v>190986</v>
+        <v>405489</v>
       </c>
       <c r="F19" t="n">
-        <v>172278</v>
+        <v>399062</v>
       </c>
       <c r="G19" t="n">
-        <v>200272</v>
+        <v>396320</v>
       </c>
       <c r="H19" t="n">
-        <v>184202</v>
+        <v>442801</v>
       </c>
       <c r="I19" t="n">
-        <v>200923</v>
+        <v>417864</v>
       </c>
       <c r="J19" t="n">
-        <v>185719</v>
+        <v>417946</v>
       </c>
       <c r="K19" t="n">
-        <v>196960</v>
+        <v>387410</v>
       </c>
       <c r="L19" t="n">
-        <v>186033</v>
+        <v>396187</v>
       </c>
       <c r="M19" t="n">
-        <v>179811</v>
+        <v>399657</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Distrito 91</t>
+          <t>Ilha da Madeira</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>47985</v>
+        <v>25252</v>
       </c>
       <c r="C20" t="n">
-        <v>47452</v>
+        <v>24161</v>
       </c>
       <c r="D20" t="n">
-        <v>150353</v>
+        <v>83639</v>
       </c>
       <c r="E20" t="n">
-        <v>141335</v>
+        <v>70322</v>
       </c>
       <c r="F20" t="n">
-        <v>135112</v>
+        <v>71740</v>
       </c>
       <c r="G20" t="n">
-        <v>146417</v>
+        <v>76996</v>
       </c>
       <c r="H20" t="n">
-        <v>138703</v>
+        <v>86500</v>
       </c>
       <c r="I20" t="n">
-        <v>156306</v>
+        <v>74164</v>
       </c>
       <c r="J20" t="n">
-        <v>161545</v>
+        <v>77249</v>
       </c>
       <c r="K20" t="n">
-        <v>148971</v>
+        <v>74178</v>
       </c>
       <c r="L20" t="n">
-        <v>163661</v>
+        <v>76780</v>
       </c>
       <c r="M20" t="n">
-        <v>158675</v>
+        <v>86460</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Distrito 12</t>
+          <t>Ilha de Porto Santo</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>28750</v>
+        <v>1005</v>
       </c>
       <c r="C21" t="n">
-        <v>31133</v>
+        <v>787</v>
       </c>
       <c r="D21" t="n">
-        <v>96156</v>
+        <v>1991</v>
       </c>
       <c r="E21" t="n">
-        <v>93479</v>
+        <v>2854</v>
       </c>
       <c r="F21" t="n">
-        <v>82990</v>
+        <v>2826</v>
       </c>
       <c r="G21" t="n">
-        <v>80639</v>
+        <v>1686</v>
       </c>
       <c r="H21" t="n">
-        <v>89399</v>
+        <v>962</v>
       </c>
       <c r="I21" t="n">
-        <v>95963</v>
+        <v>629</v>
       </c>
       <c r="J21" t="n">
-        <v>90764</v>
+        <v>1699</v>
       </c>
       <c r="K21" t="n">
-        <v>91850</v>
+        <v>1400</v>
       </c>
       <c r="L21" t="n">
-        <v>103786</v>
+        <v>2075</v>
       </c>
       <c r="M21" t="n">
-        <v>95663</v>
+        <v>2407</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Distrito 13</t>
+          <t>Ilha de Santa Maria</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>107340</v>
+        <v>3274</v>
       </c>
       <c r="C22" t="n">
-        <v>113242</v>
+        <v>1856</v>
       </c>
       <c r="D22" t="n">
-        <v>330232</v>
+        <v>10570</v>
       </c>
       <c r="E22" t="n">
-        <v>338714</v>
+        <v>8482</v>
       </c>
       <c r="F22" t="n">
-        <v>360341</v>
+        <v>4309</v>
       </c>
       <c r="G22" t="n">
-        <v>346037</v>
+        <v>7309</v>
       </c>
       <c r="H22" t="n">
-        <v>340447</v>
+        <v>6647</v>
       </c>
       <c r="I22" t="n">
-        <v>331960</v>
+        <v>7576</v>
       </c>
       <c r="J22" t="n">
-        <v>333167</v>
+        <v>6125</v>
       </c>
       <c r="K22" t="n">
-        <v>347477</v>
+        <v>10703</v>
       </c>
       <c r="L22" t="n">
-        <v>329431</v>
+        <v>6290</v>
       </c>
       <c r="M22" t="n">
-        <v>348478</v>
+        <v>8396</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Distrito 14</t>
+          <t>Ilha de São Miguel</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>57277</v>
+        <v>28695</v>
       </c>
       <c r="C23" t="n">
-        <v>56747</v>
+        <v>30617</v>
       </c>
       <c r="D23" t="n">
-        <v>198538</v>
+        <v>85884</v>
       </c>
       <c r="E23" t="n">
-        <v>168775</v>
+        <v>97699</v>
       </c>
       <c r="F23" t="n">
-        <v>179813</v>
+        <v>84765</v>
       </c>
       <c r="G23" t="n">
-        <v>186307</v>
+        <v>97335</v>
       </c>
       <c r="H23" t="n">
-        <v>198269</v>
+        <v>77979</v>
       </c>
       <c r="I23" t="n">
-        <v>173266</v>
+        <v>103467</v>
       </c>
       <c r="J23" t="n">
-        <v>167270</v>
+        <v>88305</v>
       </c>
       <c r="K23" t="n">
-        <v>196003</v>
+        <v>74410</v>
       </c>
       <c r="L23" t="n">
-        <v>177598</v>
+        <v>92715</v>
       </c>
       <c r="M23" t="n">
-        <v>170772</v>
+        <v>80270</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Distrito 15</t>
+          <t>Ilha Terceira</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>22646</v>
+        <v>11517</v>
       </c>
       <c r="C24" t="n">
-        <v>25203</v>
+        <v>12636</v>
       </c>
       <c r="D24" t="n">
-        <v>69689</v>
+        <v>32185</v>
       </c>
       <c r="E24" t="n">
-        <v>76771</v>
+        <v>34249</v>
       </c>
       <c r="F24" t="n">
-        <v>84251</v>
+        <v>33378</v>
       </c>
       <c r="G24" t="n">
-        <v>77634</v>
+        <v>33075</v>
       </c>
       <c r="H24" t="n">
-        <v>83946</v>
+        <v>36380</v>
       </c>
       <c r="I24" t="n">
-        <v>68435</v>
+        <v>40859</v>
       </c>
       <c r="J24" t="n">
-        <v>80472</v>
+        <v>33397</v>
       </c>
       <c r="K24" t="n">
-        <v>83897</v>
+        <v>35152</v>
       </c>
       <c r="L24" t="n">
-        <v>81842</v>
+        <v>49488</v>
       </c>
       <c r="M24" t="n">
-        <v>74533</v>
+        <v>49506</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Distrito 16</t>
+          <t>Ilha Graciosa</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>86084</v>
+        <v>1944</v>
       </c>
       <c r="C25" t="n">
-        <v>85910</v>
+        <v>1231</v>
       </c>
       <c r="D25" t="n">
-        <v>325287</v>
+        <v>4848</v>
       </c>
       <c r="E25" t="n">
-        <v>265964</v>
+        <v>5052</v>
       </c>
       <c r="F25" t="n">
-        <v>263424</v>
+        <v>5365</v>
       </c>
       <c r="G25" t="n">
-        <v>288513</v>
+        <v>4570</v>
       </c>
       <c r="H25" t="n">
-        <v>293656</v>
+        <v>2593</v>
       </c>
       <c r="I25" t="n">
-        <v>276578</v>
+        <v>2730</v>
       </c>
       <c r="J25" t="n">
-        <v>288957</v>
+        <v>4677</v>
       </c>
       <c r="K25" t="n">
-        <v>295905</v>
+        <v>6198</v>
       </c>
       <c r="L25" t="n">
-        <v>276817</v>
+        <v>3216</v>
       </c>
       <c r="M25" t="n">
-        <v>303974</v>
+        <v>3915</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Distrito 17</t>
+          <t>Ilha de São Jorge</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>82448</v>
+        <v>5924</v>
       </c>
       <c r="C26" t="n">
-        <v>86693</v>
+        <v>5588</v>
       </c>
       <c r="D26" t="n">
-        <v>246497</v>
+        <v>15920</v>
       </c>
       <c r="E26" t="n">
-        <v>245314</v>
+        <v>21762</v>
       </c>
       <c r="F26" t="n">
-        <v>260576</v>
+        <v>17042</v>
       </c>
       <c r="G26" t="n">
-        <v>261959</v>
+        <v>24208</v>
       </c>
       <c r="H26" t="n">
-        <v>235936</v>
+        <v>18633</v>
       </c>
       <c r="I26" t="n">
-        <v>258301</v>
+        <v>15177</v>
       </c>
       <c r="J26" t="n">
-        <v>267372</v>
+        <v>14014</v>
       </c>
       <c r="K26" t="n">
-        <v>267649</v>
+        <v>16530</v>
       </c>
       <c r="L26" t="n">
-        <v>269690</v>
+        <v>15539</v>
       </c>
       <c r="M26" t="n">
-        <v>295538</v>
+        <v>12567</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Distrito 18</t>
+          <t>Ilha do Pico</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>130124</v>
+        <v>9767</v>
       </c>
       <c r="C27" t="n">
-        <v>125511</v>
+        <v>8097</v>
       </c>
       <c r="D27" t="n">
-        <v>399668</v>
+        <v>27792</v>
       </c>
       <c r="E27" t="n">
-        <v>405489</v>
+        <v>24055</v>
       </c>
       <c r="F27" t="n">
-        <v>399062</v>
+        <v>30321</v>
       </c>
       <c r="G27" t="n">
-        <v>396320</v>
+        <v>23701</v>
       </c>
       <c r="H27" t="n">
-        <v>442801</v>
+        <v>31094</v>
       </c>
       <c r="I27" t="n">
-        <v>417864</v>
+        <v>36309</v>
       </c>
       <c r="J27" t="n">
-        <v>417946</v>
+        <v>30348</v>
       </c>
       <c r="K27" t="n">
-        <v>387410</v>
+        <v>32928</v>
       </c>
       <c r="L27" t="n">
-        <v>396187</v>
+        <v>22527</v>
       </c>
       <c r="M27" t="n">
-        <v>399657</v>
+        <v>27085</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Distrito 32</t>
+          <t>Ilha do Faial</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1005</v>
+        <v>7343</v>
       </c>
       <c r="C28" t="n">
-        <v>787</v>
+        <v>6516</v>
       </c>
       <c r="D28" t="n">
-        <v>1991</v>
+        <v>20348</v>
       </c>
       <c r="E28" t="n">
-        <v>2854</v>
+        <v>14194</v>
       </c>
       <c r="F28" t="n">
-        <v>2826</v>
+        <v>22494</v>
       </c>
       <c r="G28" t="n">
-        <v>1686</v>
+        <v>21157</v>
       </c>
       <c r="H28" t="n">
-        <v>962</v>
+        <v>16899</v>
       </c>
       <c r="I28" t="n">
-        <v>629</v>
+        <v>12910</v>
       </c>
       <c r="J28" t="n">
-        <v>1699</v>
+        <v>24087</v>
       </c>
       <c r="K28" t="n">
-        <v>1400</v>
+        <v>19260</v>
       </c>
       <c r="L28" t="n">
-        <v>2075</v>
+        <v>19641</v>
       </c>
       <c r="M28" t="n">
-        <v>2407</v>
+        <v>18907</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Distrito 42</t>
+          <t>Ilha das Flores</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>28695</v>
+        <v>3327</v>
       </c>
       <c r="C29" t="n">
-        <v>30617</v>
+        <v>4526</v>
       </c>
       <c r="D29" t="n">
-        <v>85884</v>
+        <v>16545</v>
       </c>
       <c r="E29" t="n">
-        <v>97699</v>
+        <v>14076</v>
       </c>
       <c r="F29" t="n">
-        <v>84765</v>
+        <v>10552</v>
       </c>
       <c r="G29" t="n">
-        <v>97335</v>
+        <v>13703</v>
       </c>
       <c r="H29" t="n">
-        <v>77979</v>
+        <v>9816</v>
       </c>
       <c r="I29" t="n">
-        <v>103467</v>
+        <v>10192</v>
       </c>
       <c r="J29" t="n">
-        <v>88305</v>
+        <v>17223</v>
       </c>
       <c r="K29" t="n">
-        <v>74410</v>
+        <v>12506</v>
       </c>
       <c r="L29" t="n">
-        <v>92715</v>
+        <v>12607</v>
       </c>
       <c r="M29" t="n">
-        <v>80270</v>
+        <v>19283</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Distrito 43</t>
+          <t>Ilha do Corvo</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>11517</v>
+        <v>841</v>
       </c>
       <c r="C30" t="n">
-        <v>12636</v>
+        <v>1017</v>
       </c>
       <c r="D30" t="n">
-        <v>32185</v>
+        <v>2163</v>
       </c>
       <c r="E30" t="n">
-        <v>34249</v>
+        <v>3695</v>
       </c>
       <c r="F30" t="n">
-        <v>33378</v>
+        <v>3447</v>
       </c>
       <c r="G30" t="n">
-        <v>33075</v>
+        <v>1276</v>
       </c>
       <c r="H30" t="n">
-        <v>36380</v>
+        <v>334</v>
       </c>
       <c r="I30" t="n">
-        <v>40859</v>
+        <v>3711</v>
       </c>
       <c r="J30" t="n">
-        <v>33397</v>
+        <v>1766</v>
       </c>
       <c r="K30" t="n">
-        <v>35152</v>
+        <v>2991</v>
       </c>
       <c r="L30" t="n">
-        <v>49488</v>
+        <v>397</v>
       </c>
       <c r="M30" t="n">
-        <v>49506</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Distrito 44</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>1944</v>
-      </c>
-      <c r="C31" t="n">
-        <v>1231</v>
-      </c>
-      <c r="D31" t="n">
-        <v>4848</v>
-      </c>
-      <c r="E31" t="n">
-        <v>5052</v>
-      </c>
-      <c r="F31" t="n">
-        <v>5365</v>
-      </c>
-      <c r="G31" t="n">
-        <v>4570</v>
-      </c>
-      <c r="H31" t="n">
-        <v>2593</v>
-      </c>
-      <c r="I31" t="n">
-        <v>2730</v>
-      </c>
-      <c r="J31" t="n">
-        <v>4677</v>
-      </c>
-      <c r="K31" t="n">
-        <v>6198</v>
-      </c>
-      <c r="L31" t="n">
-        <v>3216</v>
-      </c>
-      <c r="M31" t="n">
-        <v>3915</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Distrito 45</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>5924</v>
-      </c>
-      <c r="C32" t="n">
-        <v>5588</v>
-      </c>
-      <c r="D32" t="n">
-        <v>15920</v>
-      </c>
-      <c r="E32" t="n">
-        <v>21762</v>
-      </c>
-      <c r="F32" t="n">
-        <v>17042</v>
-      </c>
-      <c r="G32" t="n">
-        <v>24208</v>
-      </c>
-      <c r="H32" t="n">
-        <v>18633</v>
-      </c>
-      <c r="I32" t="n">
-        <v>15177</v>
-      </c>
-      <c r="J32" t="n">
-        <v>14014</v>
-      </c>
-      <c r="K32" t="n">
-        <v>16530</v>
-      </c>
-      <c r="L32" t="n">
-        <v>15539</v>
-      </c>
-      <c r="M32" t="n">
-        <v>12567</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Distrito 46</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>9767</v>
-      </c>
-      <c r="C33" t="n">
-        <v>8097</v>
-      </c>
-      <c r="D33" t="n">
-        <v>27792</v>
-      </c>
-      <c r="E33" t="n">
-        <v>24055</v>
-      </c>
-      <c r="F33" t="n">
-        <v>30321</v>
-      </c>
-      <c r="G33" t="n">
-        <v>23701</v>
-      </c>
-      <c r="H33" t="n">
-        <v>31094</v>
-      </c>
-      <c r="I33" t="n">
-        <v>36309</v>
-      </c>
-      <c r="J33" t="n">
-        <v>30348</v>
-      </c>
-      <c r="K33" t="n">
-        <v>32928</v>
-      </c>
-      <c r="L33" t="n">
-        <v>22527</v>
-      </c>
-      <c r="M33" t="n">
-        <v>27085</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Distrito 47</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>7343</v>
-      </c>
-      <c r="C34" t="n">
-        <v>6516</v>
-      </c>
-      <c r="D34" t="n">
-        <v>20348</v>
-      </c>
-      <c r="E34" t="n">
-        <v>14194</v>
-      </c>
-      <c r="F34" t="n">
-        <v>22494</v>
-      </c>
-      <c r="G34" t="n">
-        <v>21157</v>
-      </c>
-      <c r="H34" t="n">
-        <v>16899</v>
-      </c>
-      <c r="I34" t="n">
-        <v>12910</v>
-      </c>
-      <c r="J34" t="n">
-        <v>24087</v>
-      </c>
-      <c r="K34" t="n">
-        <v>19260</v>
-      </c>
-      <c r="L34" t="n">
-        <v>19641</v>
-      </c>
-      <c r="M34" t="n">
-        <v>18907</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Distrito 48</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>3327</v>
-      </c>
-      <c r="C35" t="n">
-        <v>4526</v>
-      </c>
-      <c r="D35" t="n">
-        <v>16545</v>
-      </c>
-      <c r="E35" t="n">
-        <v>14076</v>
-      </c>
-      <c r="F35" t="n">
-        <v>10552</v>
-      </c>
-      <c r="G35" t="n">
-        <v>13703</v>
-      </c>
-      <c r="H35" t="n">
-        <v>9816</v>
-      </c>
-      <c r="I35" t="n">
-        <v>10192</v>
-      </c>
-      <c r="J35" t="n">
-        <v>17223</v>
-      </c>
-      <c r="K35" t="n">
-        <v>12506</v>
-      </c>
-      <c r="L35" t="n">
-        <v>12607</v>
-      </c>
-      <c r="M35" t="n">
-        <v>19283</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Distrito 49</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>841</v>
-      </c>
-      <c r="C36" t="n">
-        <v>1017</v>
-      </c>
-      <c r="D36" t="n">
-        <v>2163</v>
-      </c>
-      <c r="E36" t="n">
-        <v>3695</v>
-      </c>
-      <c r="F36" t="n">
-        <v>3447</v>
-      </c>
-      <c r="G36" t="n">
-        <v>1276</v>
-      </c>
-      <c r="H36" t="n">
-        <v>334</v>
-      </c>
-      <c r="I36" t="n">
-        <v>3711</v>
-      </c>
-      <c r="J36" t="n">
-        <v>1766</v>
-      </c>
-      <c r="K36" t="n">
-        <v>2991</v>
-      </c>
-      <c r="L36" t="n">
-        <v>397</v>
-      </c>
-      <c r="M36" t="n">
         <v>1979</v>
       </c>
     </row>

</xml_diff>